<commit_message>
Record owner approval, integrated impact graph and complete close-review QA
</commit_message>
<xml_diff>
--- a/docs/legal/gap-instruments/case-briefs/qa/cold-start/evidence-proposal/tracker.xlsx
+++ b/docs/legal/gap-instruments/case-briefs/qa/cold-start/evidence-proposal/tracker.xlsx
@@ -355,7 +355,7 @@
     <t>State SHA-256</t>
   </si>
   <si>
-    <t>1ec7f499d1ad9f560683c7aef48dee4b300af82bf8ebdfbb725a5ea60bd2d947</t>
+    <t>9e7a55d20aae25fb6a95fdf4aa92796cee32dcf87623a577b8972ad3f6f32a4f</t>
   </si>
   <si>
     <t>docs/finance/evidence/SH-FIN-HUMAN-001/source.json</t>
@@ -367,7 +367,7 @@
     <t>docs/legal/gap-instruments/period-close/README.md</t>
   </si>
   <si>
-    <t>1f764afff496bd216dfca3fd1ffac4accf7433cf0404557f894312f82887577a</t>
+    <t>2cf05a38cb0a634ba8355e6f5e046977ada35dad0a83d210b7cd265491c59e20</t>
   </si>
   <si>
     <t>docs/legal/gap-instruments/period-close/case.json</t>

</xml_diff>